<commit_message>
numerous changes to file structure
</commit_message>
<xml_diff>
--- a/descriptives/micro_descriptives.xlsx
+++ b/descriptives/micro_descriptives.xlsx
@@ -620,22 +620,22 @@
         <v>215852</v>
       </c>
       <c r="D6" t="n">
-        <v>28737.37359742307</v>
+        <v>27592.06718082844</v>
       </c>
       <c r="E6" t="n">
-        <v>282253.3517800478</v>
+        <v>286630.509705687</v>
       </c>
       <c r="F6" t="n">
-        <v>2.454000000000001</v>
+        <v>2.454</v>
       </c>
       <c r="G6" t="n">
-        <v>2.945708</v>
+        <v>2.945707999999999</v>
       </c>
       <c r="H6" t="n">
         <v>13646.88768230084</v>
       </c>
       <c r="I6" t="n">
-        <v>13726.51732133783</v>
+        <v>13726.51732133782</v>
       </c>
       <c r="J6" t="n">
         <v>14.13816113913604</v>
@@ -883,10 +883,10 @@
         <v>212363</v>
       </c>
       <c r="E2" t="n">
-        <v>22459.17139498537</v>
+        <v>22344.6407533259</v>
       </c>
       <c r="F2" t="n">
-        <v>261780.5335380293</v>
+        <v>262218.2493305932</v>
       </c>
       <c r="G2" t="n">
         <v>3.663974800000001</v>
@@ -926,7 +926,7 @@
         <v>275606.8031777889</v>
       </c>
       <c r="G3" t="n">
-        <v>2.914845000000001</v>
+        <v>2.914845</v>
       </c>
       <c r="H3" t="n">
         <v>3.1242295</v>
@@ -938,7 +938,7 @@
         <v>15711.33188918279</v>
       </c>
       <c r="K3" t="n">
-        <v>14.29482412342049</v>
+        <v>14.29482412342048</v>
       </c>
     </row>
     <row r="4">
@@ -957,10 +957,10 @@
         <v>31687.0539775754</v>
       </c>
       <c r="E4" t="n">
-        <v>7930.017260423305</v>
+        <v>7836.993381324715</v>
       </c>
       <c r="F4" t="n">
-        <v>62210.7923959368</v>
+        <v>62385.99673037831</v>
       </c>
       <c r="G4" t="n">
         <v>2.293214645516241</v>

</xml_diff>